<commit_message>
Fim dos ajustes nos teste de escala e inicio dos testes de reescala
Fim dos ajustes nos teste de escala e inicio dos testes de reescala
</commit_message>
<xml_diff>
--- a/algoritmoGeneticoReescala/melhor_escala_ag.xlsx
+++ b/algoritmoGeneticoReescala/melhor_escala_ag.xlsx
@@ -772,11 +772,11 @@
       <c r="AA2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC2" s="5" t="n">
-        <v>0</v>
+      <c r="AB2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
@@ -997,11 +997,11 @@
       <c r="AB4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD4" s="5" t="n">
-        <v>0</v>
+      <c r="AC4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AE4" s="5" t="n">
         <v>0</v>
@@ -1054,11 +1054,11 @@
       <c r="J5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" s="5" t="n">
-        <v>0</v>
+      <c r="K5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>0</v>
@@ -1153,17 +1153,17 @@
       <c r="F6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>1</v>
+      <c r="G6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="K6" s="5" t="n">
         <v>0</v>
@@ -1288,11 +1288,11 @@
       <c r="N7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="O7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="4" t="n">
-        <v>1</v>
+      <c r="O7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1381,44 +1381,44 @@
       <c r="H8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U8" s="5" t="n">
-        <v>0</v>
+      <c r="I8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="V8" s="5" t="n">
         <v>0</v>
@@ -1429,38 +1429,38 @@
       <c r="X8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI8" s="5" t="n">
-        <v>0</v>
+      <c r="Y8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1489,17 +1489,17 @@
       <c r="G9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>1</v>
+      <c r="H9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L9" s="5" t="n">
         <v>0</v>
@@ -1549,14 +1549,14 @@
       <c r="AA9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD9" s="4" t="n">
-        <v>1</v>
+      <c r="AB9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AE9" s="5" t="n">
         <v>0</v>
@@ -1603,14 +1603,14 @@
       <c r="H10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>1</v>
+      <c r="I10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L10" s="5" t="n">
         <v>0</v>
@@ -1633,11 +1633,11 @@
       <c r="R10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>1</v>
+      <c r="S10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U10" s="5" t="n">
         <v>0</v>
@@ -1648,11 +1648,11 @@
       <c r="W10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="X10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y10" s="5" t="n">
-        <v>0</v>
+      <c r="X10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="Z10" s="5" t="n">
         <v>0</v>
@@ -1705,11 +1705,11 @@
       <c r="E11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>0</v>
+      <c r="F11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="H11" s="5" t="n">
         <v>0</v>
@@ -1732,11 +1732,11 @@
       <c r="N11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="O11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P11" s="5" t="n">
-        <v>0</v>
+      <c r="O11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1747,11 +1747,11 @@
       <c r="S11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U11" s="5" t="n">
-        <v>0</v>
+      <c r="T11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="V11" s="5" t="n">
         <v>0</v>
@@ -1780,20 +1780,20 @@
       <c r="AD11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AE11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI11" s="4" t="n">
-        <v>1</v>
+      <c r="AE11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI11" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1834,11 +1834,11 @@
       <c r="K12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>1</v>
+      <c r="L12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="N12" s="5" t="n">
         <v>0</v>
@@ -1873,38 +1873,38 @@
       <c r="X12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI12" s="5" t="n">
-        <v>0</v>
+      <c r="Y12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI12" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1948,17 +1948,17 @@
       <c r="L13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P13" s="5" t="n">
-        <v>0</v>
+      <c r="M13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1969,23 +1969,23 @@
       <c r="S13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y13" s="5" t="n">
-        <v>0</v>
+      <c r="T13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="Z13" s="5" t="n">
         <v>0</v>
@@ -1996,26 +1996,26 @@
       <c r="AB13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI13" s="4" t="n">
-        <v>1</v>
+      <c r="AC13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI13" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2119,14 +2119,14 @@
       <c r="AF14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AG14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI14" s="5" t="n">
-        <v>0</v>
+      <c r="AG14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI14" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2158,11 +2158,11 @@
       <c r="H15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="4" t="n">
-        <v>1</v>
+      <c r="I15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="K15" s="5" t="n">
         <v>0</v>
@@ -2191,11 +2191,11 @@
       <c r="S15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U15" s="5" t="n">
-        <v>0</v>
+      <c r="T15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="V15" s="5" t="n">
         <v>0</v>
@@ -2272,23 +2272,23 @@
       <c r="I16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O16" s="5" t="n">
-        <v>0</v>
+      <c r="J16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="P16" s="5" t="n">
         <v>0</v>
@@ -2329,26 +2329,26 @@
       <c r="AB16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI16" s="4" t="n">
-        <v>1</v>
+      <c r="AC16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI16" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -2392,74 +2392,74 @@
       <c r="L17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="X17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC17" s="4" t="n">
-        <v>1</v>
+      <c r="M17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC17" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AD17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AE17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI17" s="5" t="n">
-        <v>0</v>
+      <c r="AE17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI17" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -2608,56 +2608,56 @@
       <c r="J19" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA19" s="5" t="n">
-        <v>0</v>
+      <c r="K19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AB19" s="5" t="n">
         <v>0</v>
@@ -2860,26 +2860,26 @@
       <c r="T21" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="X21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="4" t="n">
-        <v>1</v>
+      <c r="U21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA21" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AB21" s="5" t="n">
         <v>0</v>
@@ -2941,11 +2941,11 @@
       <c r="J22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="5" t="n">
-        <v>0</v>
+      <c r="K22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="M22" s="5" t="n">
         <v>0</v>
@@ -2956,11 +2956,11 @@
       <c r="O22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="P22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q22" s="5" t="n">
-        <v>0</v>
+      <c r="P22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R22" s="5" t="n">
         <v>0</v>
@@ -3037,11 +3037,11 @@
       <c r="E23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="4" t="n">
-        <v>1</v>
+      <c r="F23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="H23" s="5" t="n">
         <v>0</v>
@@ -3118,14 +3118,14 @@
       <c r="AF23" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AG23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI23" s="4" t="n">
-        <v>1</v>
+      <c r="AG23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI23" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -3154,11 +3154,11 @@
       <c r="G24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="4" t="n">
-        <v>1</v>
+      <c r="H24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>0</v>
@@ -3229,14 +3229,14 @@
       <c r="AF24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AG24" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI24" s="4" t="n">
-        <v>1</v>
+      <c r="AG24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI24" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -3289,11 +3289,11 @@
       <c r="O25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="P25" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q25" s="5" t="n">
-        <v>0</v>
+      <c r="P25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="R25" s="5" t="n">
         <v>0</v>
@@ -3436,11 +3436,11 @@
       <c r="AA26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC26" s="4" t="n">
-        <v>1</v>
+      <c r="AB26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC26" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AD26" s="5" t="n">
         <v>0</v>
@@ -3511,50 +3511,50 @@
       <c r="O27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="P27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="X27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD27" s="5" t="n">
-        <v>0</v>
+      <c r="P27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AE27" s="5" t="n">
         <v>0</v>
@@ -3565,11 +3565,11 @@
       <c r="AG27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI27" s="5" t="n">
-        <v>0</v>
+      <c r="AH27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI27" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -3601,74 +3601,74 @@
       <c r="H28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="X28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE28" s="4" t="n">
-        <v>1</v>
+      <c r="I28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE28" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AF28" s="5" t="n">
         <v>0</v>
@@ -3709,17 +3709,17 @@
       <c r="G29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" s="4" t="n">
-        <v>1</v>
+      <c r="H29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L29" s="5" t="n">
         <v>0</v>
@@ -3757,29 +3757,29 @@
       <c r="W29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="X29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE29" s="5" t="n">
-        <v>0</v>
+      <c r="X29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AF29" s="5" t="n">
         <v>0</v>
@@ -3856,14 +3856,14 @@
       <c r="S30" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V30" s="4" t="n">
-        <v>1</v>
+      <c r="T30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V30" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="W30" s="5" t="n">
         <v>0</v>
@@ -3880,29 +3880,29 @@
       <c r="AA30" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AB30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI30" s="4" t="n">
-        <v>1</v>
+      <c r="AB30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI30" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -3937,11 +3937,11 @@
       <c r="I31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K31" s="5" t="n">
-        <v>0</v>
+      <c r="J31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="L31" s="5" t="n">
         <v>0</v>
@@ -3958,17 +3958,17 @@
       <c r="P31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T31" s="4" t="n">
-        <v>1</v>
+      <c r="Q31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T31" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U31" s="5" t="n">
         <v>0</v>
@@ -4042,44 +4042,44 @@
       <c r="G32" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T32" s="4" t="n">
-        <v>1</v>
+      <c r="H32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T32" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U32" s="5" t="n">
         <v>0</v>
@@ -4114,17 +4114,17 @@
       <c r="AE32" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AF32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH32" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI32" s="5" t="n">
-        <v>0</v>
+      <c r="AF32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI32" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -4150,44 +4150,44 @@
       <c r="F33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S33" s="4" t="n">
-        <v>1</v>
+      <c r="G33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T33" s="5" t="n">
         <v>0</v>
@@ -4327,11 +4327,11 @@
       <c r="AB34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AC34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD34" s="4" t="n">
-        <v>1</v>
+      <c r="AC34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD34" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AE34" s="5" t="n">
         <v>0</v>
@@ -4342,11 +4342,11 @@
       <c r="AG34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH34" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI34" s="5" t="n">
-        <v>0</v>
+      <c r="AH34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI34" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -4411,17 +4411,17 @@
       <c r="S35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W35" s="5" t="n">
-        <v>0</v>
+      <c r="T35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="X35" s="5" t="n">
         <v>0</v>
@@ -4432,14 +4432,14 @@
       <c r="Z35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AA35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC35" s="5" t="n">
-        <v>0</v>
+      <c r="AA35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AD35" s="5" t="n">
         <v>0</v>
@@ -4507,20 +4507,20 @@
       <c r="N36" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="O36" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S36" s="4" t="n">
-        <v>1</v>
+      <c r="O36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T36" s="5" t="n">
         <v>0</v>
@@ -4594,11 +4594,11 @@
       <c r="F37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="5" t="n">
-        <v>0</v>
+      <c r="G37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="I37" s="5" t="n">
         <v>0</v>
@@ -4738,11 +4738,11 @@
       <c r="Q38" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S38" s="4" t="n">
-        <v>1</v>
+      <c r="R38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S38" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T38" s="5" t="n">
         <v>0</v>
@@ -4819,11 +4819,11 @@
       <c r="G39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I39" s="5" t="n">
-        <v>0</v>
+      <c r="H39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="J39" s="5" t="n">
         <v>0</v>
@@ -4834,11 +4834,11 @@
       <c r="L39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="M39" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N39" s="5" t="n">
-        <v>0</v>
+      <c r="M39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="O39" s="5" t="n">
         <v>0</v>
@@ -4942,11 +4942,11 @@
       <c r="K40" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="L40" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M40" s="5" t="n">
-        <v>0</v>
+      <c r="L40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="N40" s="5" t="n">
         <v>0</v>
@@ -5035,11 +5035,11 @@
       <c r="E41" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="4" t="n">
-        <v>1</v>
+      <c r="F41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="H41" s="5" t="n">
         <v>0</v>
@@ -5071,20 +5071,20 @@
       <c r="Q41" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="R41" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T41" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V41" s="4" t="n">
-        <v>1</v>
+      <c r="R41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V41" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="W41" s="5" t="n">
         <v>0</v>
@@ -5113,11 +5113,11 @@
       <c r="AE41" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AF41" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG41" s="5" t="n">
-        <v>0</v>
+      <c r="AF41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG41" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AH41" s="5" t="n">
         <v>0</v>
@@ -5188,53 +5188,53 @@
       <c r="S42" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI42" s="5" t="n">
-        <v>0</v>
+      <c r="T42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI42" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -5302,8 +5302,8 @@
       <c r="T43" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U43" s="4" t="n">
-        <v>1</v>
+      <c r="U43" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="V43" s="5" t="n">
         <v>0</v>
@@ -5332,20 +5332,20 @@
       <c r="AD43" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AE43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF43" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH43" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI43" s="5" t="n">
-        <v>0</v>
+      <c r="AE43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI43" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -5395,20 +5395,20 @@
       <c r="N44" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="O44" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P44" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q44" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R44" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S44" s="4" t="n">
-        <v>1</v>
+      <c r="O44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S44" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T44" s="5" t="n">
         <v>0</v>
@@ -5509,17 +5509,17 @@
       <c r="O45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="P45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S45" s="4" t="n">
-        <v>1</v>
+      <c r="P45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S45" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T45" s="5" t="n">
         <v>0</v>
@@ -5536,11 +5536,11 @@
       <c r="X45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Y45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z45" s="5" t="n">
-        <v>0</v>
+      <c r="Y45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AA45" s="5" t="n">
         <v>0</v>
@@ -5557,17 +5557,17 @@
       <c r="AE45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AF45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI45" s="4" t="n">
-        <v>1</v>
+      <c r="AF45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI45" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -5620,20 +5620,20 @@
       <c r="O46" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="P46" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q46" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R46" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S46" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T46" s="4" t="n">
-        <v>1</v>
+      <c r="P46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T46" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U46" s="5" t="n">
         <v>0</v>
@@ -5704,11 +5704,11 @@
       <c r="F47" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="4" t="n">
-        <v>1</v>
+      <c r="G47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="I47" s="5" t="n">
         <v>0</v>
@@ -5725,11 +5725,11 @@
       <c r="M47" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O47" s="4" t="n">
-        <v>1</v>
+      <c r="N47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O47" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="P47" s="5" t="n">
         <v>0</v>
@@ -5746,50 +5746,50 @@
       <c r="T47" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="U47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="X47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI47" s="4" t="n">
-        <v>1</v>
+      <c r="U47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI47" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -5857,29 +5857,29 @@
       <c r="T48" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="U48" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V48" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W48" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="X48" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y48" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z48" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA48" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB48" s="5" t="n">
-        <v>0</v>
+      <c r="U48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W48" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y48" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB48" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="AC48" s="5" t="n">
         <v>0</v>
@@ -5896,8 +5896,8 @@
       <c r="AG48" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AH48" s="4" t="n">
-        <v>1</v>
+      <c r="AH48" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AI48" s="5" t="n">
         <v>0</v>
@@ -5935,11 +5935,11 @@
       <c r="I49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="J49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K49" s="4" t="n">
-        <v>1</v>
+      <c r="J49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="L49" s="5" t="n">
         <v>0</v>
@@ -5956,17 +5956,17 @@
       <c r="P49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Q49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T49" s="5" t="n">
-        <v>0</v>
+      <c r="Q49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="U49" s="5" t="n">
         <v>0</v>
@@ -5983,20 +5983,20 @@
       <c r="Y49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC49" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD49" s="4" t="n">
-        <v>1</v>
+      <c r="Z49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD49" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="AE49" s="5" t="n">
         <v>0</v>
@@ -6034,50 +6034,50 @@
       <c r="E50" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G50" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I50" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K50" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M50" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O50" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q50" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S50" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T50" s="4" t="n">
-        <v>1</v>
+      <c r="F50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T50" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U50" s="5" t="n">
         <v>0</v>
@@ -6226,14 +6226,14 @@
       <c r="AF51" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AG51" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH51" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI51" s="4" t="n">
-        <v>1</v>
+      <c r="AG51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH51" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI51" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -6280,26 +6280,26 @@
       <c r="M52" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N52" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O52" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P52" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q52" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R52" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S52" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T52" s="4" t="n">
-        <v>1</v>
+      <c r="N52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T52" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="U52" s="5" t="n">
         <v>0</v>

</xml_diff>